<commit_message>
feat: sync item drop catalog excel with full boss and growth balance
</commit_message>
<xml_diff>
--- a/public/downloads/soongsil_rpg_item_drops_catalog.xlsx
+++ b/public/downloads/soongsil_rpg_item_drops_catalog.xlsx
@@ -7,6 +7,7 @@
     <sheet name="운동장_몬스터드랍" sheetId="2" r:id="rId2"/>
     <sheet name="보스레이드_전리품" sheetId="3" r:id="rId3"/>
     <sheet name="제작대_조합레시피" sheetId="4" r:id="rId4"/>
+    <sheet name="성장곡선_스펙밸런스" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -400,16 +401,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H26"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="32.83203125" customWidth="1"/>
-    <col min="7" max="7" width="48.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
+    <col min="7" max="7" width="54.83203125" customWidth="1"/>
+    <col min="8" max="8" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -648,391 +649,470 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>item_red_potion</v>
+        <v>item_perfect_exam</v>
       </c>
       <c r="B10" t="str">
-        <v>🍷</v>
+        <v>💯</v>
       </c>
       <c r="C10" t="str">
-        <v>빨간 물약</v>
+        <v>백점만점 시험지</v>
       </c>
       <c r="D10" t="str">
-        <v>소비품</v>
+        <v>재료</v>
       </c>
       <c r="E10" t="str">
-        <v>즉시 회복</v>
+        <v>이벤트 전리품</v>
       </c>
       <c r="F10" t="str">
-        <v>체력(HP) +10 즉시 회복</v>
+        <v>📚 시험의 제왕 호칭 교환 재료</v>
       </c>
       <c r="G10" t="str">
-        <v>복도 제작(허브 1+5G), 보스전 드랍</v>
+        <v>😈 중간고사 대마왕 토벌(100% 확정)</v>
       </c>
       <c r="H10" t="str">
-        <v>가장 기본적인 휴대용 회복 물약</v>
+        <v>매점 호칭 교환소에서 [📚 시험의 제왕] 호칭 교환용</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>item_orange_potion</v>
+        <v>item_eval_paper</v>
       </c>
       <c r="B11" t="str">
-        <v>🧪</v>
+        <v>📜</v>
       </c>
       <c r="C11" t="str">
-        <v>주황 물약</v>
+        <v>A+ 만점 수행평가지</v>
       </c>
       <c r="D11" t="str">
-        <v>소비품</v>
+        <v>재료</v>
       </c>
       <c r="E11" t="str">
-        <v>즉시 회복</v>
+        <v>보스 전리품</v>
       </c>
       <c r="F11" t="str">
-        <v>체력(HP) +25 즉시 회복</v>
+        <v>수행평가 만점 증표 · 매점 매각 25G</v>
       </c>
       <c r="G11" t="str">
-        <v>복도 제작(허브 2+개나리 1+10G), 보스전 드랍</v>
+        <v>🐕 수행평가 3두마수 케르베로스 토벌(100% 확정)</v>
       </c>
       <c r="H11" t="str">
-        <v>중급 체력 회복 물약으로 필드 전투 생존율 극대화</v>
+        <v>케르베로스 전용 전리품 (매점 매각 시 25G 환전 가능)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>item_revive_scroll</v>
+        <v>item_red_potion</v>
       </c>
       <c r="B12" t="str">
-        <v>📜</v>
+        <v>🍷</v>
       </c>
       <c r="C12" t="str">
-        <v>부활 주문서</v>
+        <v>빨간 물약</v>
       </c>
       <c r="D12" t="str">
         <v>소비품</v>
       </c>
       <c r="E12" t="str">
-        <v>부활 주문</v>
+        <v>즉시 회복</v>
       </c>
       <c r="F12" t="str">
-        <v>쓰러진 동료 50% HP 부활</v>
+        <v>체력(HP) +10 즉시 회복</v>
       </c>
       <c r="G12" t="str">
-        <v>복도 제작(허브 3+은행잎 1+25G)</v>
+        <v>복도 제작(허브 1+5G), 보스전 드랍</v>
       </c>
       <c r="H12" t="str">
-        <v>보스 레이드 중 사망한 급우를 부활시키는 파티 필수템</v>
+        <v>가장 기본적인 휴대용 회복 물약</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>equip_wood_sword</v>
+        <v>item_orange_potion</v>
       </c>
       <c r="B13" t="str">
-        <v>🗡️</v>
+        <v>🧪</v>
       </c>
       <c r="C13" t="str">
-        <v>나무검</v>
+        <v>주홍 물약</v>
       </c>
       <c r="D13" t="str">
-        <v>장비</v>
+        <v>소비품</v>
       </c>
       <c r="E13" t="str">
-        <v>무기 (Weapon)</v>
+        <v>즉시 회복</v>
       </c>
       <c r="F13" t="str">
-        <v>공격력(ATK) +15</v>
+        <v>체력(HP) +25 즉시 회복</v>
       </c>
       <c r="G13" t="str">
-        <v>복도 제작(목재 10+15G), 숭실이 선물</v>
+        <v>복도 제작(허브 2+개나리 1+10G), 보스전 드랍</v>
       </c>
       <c r="H13" t="str">
-        <v>1학년 신입생 입학 기본 무기 (1티어)</v>
+        <v>중급 체력 회복 물약으로 필드 전투 생존율 극대화</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>equip_wood_helmet</v>
+        <v>item_revive_scroll</v>
       </c>
       <c r="B14" t="str">
-        <v>🪖</v>
+        <v>📜</v>
       </c>
       <c r="C14" t="str">
-        <v>나무투구</v>
+        <v>부활 주문서</v>
       </c>
       <c r="D14" t="str">
-        <v>장비</v>
+        <v>소비품</v>
       </c>
       <c r="E14" t="str">
-        <v>투구 (Helmet)</v>
+        <v>부활 주문</v>
       </c>
       <c r="F14" t="str">
-        <v>방어력(DEF) +8, 체력(HP) +25</v>
+        <v>쓰러진 동료 50% HP 부활</v>
       </c>
       <c r="G14" t="str">
-        <v>복도 제작(목재 10+15G), 골렘 드랍(25%)</v>
+        <v>복도 제작(허브 3+은행잎 1+25G)</v>
       </c>
       <c r="H14" t="str">
-        <v>1학년 1반 기본 방어구 (1티어)</v>
+        <v>보스 레이드 중 사망한 급우를 부활시키는 파티 필수템</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>equip_wood_armor</v>
+        <v>equip_wood_sword</v>
       </c>
       <c r="B15" t="str">
-        <v>🛡️</v>
+        <v>🗡️</v>
       </c>
       <c r="C15" t="str">
-        <v>나무갑옷</v>
+        <v>나무검</v>
       </c>
       <c r="D15" t="str">
         <v>장비</v>
       </c>
       <c r="E15" t="str">
-        <v>갑옷 (Armor)</v>
+        <v>무기 (Weapon)</v>
       </c>
       <c r="F15" t="str">
-        <v>방어력(DEF) +15, 체력(HP) +15</v>
+        <v>공격력(ATK) +15</v>
       </c>
       <c r="G15" t="str">
-        <v>복도 제작(목재 10+20G), 골렘 드랍(25%)</v>
+        <v>복도 제작(목재 10+15G), 숭실이 선물</v>
       </c>
       <c r="H15" t="str">
-        <v>1학년 1반 기본 방어구 (1티어)</v>
+        <v>1학년 신입생 입학 기본 무기 (1티어)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>equip_leather_sword</v>
+        <v>equip_wood_helmet</v>
       </c>
       <c r="B16" t="str">
-        <v>🗡️</v>
+        <v>🪖</v>
       </c>
       <c r="C16" t="str">
-        <v>가죽손잡이 세이버</v>
+        <v>나무투구</v>
       </c>
       <c r="D16" t="str">
         <v>장비</v>
       </c>
       <c r="E16" t="str">
-        <v>무기 (Weapon)</v>
+        <v>투구 (Helmet)</v>
       </c>
       <c r="F16" t="str">
-        <v>공격력(ATK) +20</v>
+        <v>방어력(DEF) +8, 체력(HP) +25</v>
       </c>
       <c r="G16" t="str">
-        <v>복도 제작(보스가죽 1+농구가죽 10+풋살가죽 10+35G), 골키퍼(5%), 골렘(15%)</v>
+        <v>복도 제작(목재 10+15G), 골렘 드랍(25%)</v>
       </c>
       <c r="H16" t="str">
-        <v>2티어 실전 검</v>
+        <v>1학년 1반 기본 방어구 (1티어)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>equip_leather_helmet</v>
+        <v>equip_wood_armor</v>
       </c>
       <c r="B17" t="str">
-        <v>⛑️</v>
+        <v>🛡️</v>
       </c>
       <c r="C17" t="str">
-        <v>가죽투구</v>
+        <v>나무갑옷</v>
       </c>
       <c r="D17" t="str">
         <v>장비</v>
       </c>
       <c r="E17" t="str">
-        <v>투구 (Helmet)</v>
+        <v>갑옷 (Armor)</v>
       </c>
       <c r="F17" t="str">
-        <v>방어력(DEF) +12, 체력(HP) +28</v>
+        <v>방어력(DEF) +15, 체력(HP) +15</v>
       </c>
       <c r="G17" t="str">
-        <v>복도 제작(보스가죽 1+풋살가죽 20+40G), 골키퍼(8%)</v>
+        <v>복도 제작(목재 10+20G), 골렘 드랍(25%)</v>
       </c>
       <c r="H17" t="str">
-        <v>2티어 스포츠 방어구</v>
+        <v>1학년 1반 기본 방어구 (1티어)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>equip_leather_armor</v>
+        <v>equip_leather_sword</v>
       </c>
       <c r="B18" t="str">
-        <v>🥋</v>
+        <v>🗡️</v>
       </c>
       <c r="C18" t="str">
-        <v>가죽갑옷</v>
+        <v>가죽손잡이 세이버</v>
       </c>
       <c r="D18" t="str">
         <v>장비</v>
       </c>
       <c r="E18" t="str">
-        <v>갑옷 (Armor)</v>
+        <v>무기 (Weapon)</v>
       </c>
       <c r="F18" t="str">
-        <v>방어력(DEF) +17, 체력(HP) +20</v>
+        <v>공격력(ATK) +20</v>
       </c>
       <c r="G18" t="str">
-        <v>복도 제작(보스가죽 1+농구가죽 30+50G), 림가디언(8%)</v>
+        <v>복도 제작(보스가죽 1+농구가죽 10+풋살가죽 10+35G), 골키퍼(5%), 골렘(15%)</v>
       </c>
       <c r="H18" t="str">
-        <v>2티어 스포츠 방어구</v>
+        <v>2티어 실전 검</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>equip_forsythia_ring</v>
+        <v>equip_leather_helmet</v>
       </c>
       <c r="B19" t="str">
-        <v>🌼</v>
+        <v>⛑️</v>
       </c>
       <c r="C19" t="str">
-        <v>성실의 개나리 반지</v>
+        <v>가죽투구</v>
       </c>
       <c r="D19" t="str">
         <v>장비</v>
       </c>
       <c r="E19" t="str">
-        <v>장신구 (Accessory)</v>
+        <v>투구 (Helmet)</v>
       </c>
       <c r="F19" t="str">
-        <v>ATK +10, DEF +10, HP +20</v>
+        <v>방어력(DEF) +12, 체력(HP) +28</v>
       </c>
       <c r="G19" t="str">
-        <v>복도 제작(개나리 20+30G), 보스 레이드(5%)</v>
+        <v>복도 제작(보스가죽 1+풋살가죽 20+40G), 골키퍼(8%)</v>
       </c>
       <c r="H19" t="str">
-        <v>숭실의 교화 개나리의 성실한 빛이 담긴 반지</v>
+        <v>2티어 스포츠 방어구</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>equip_ginkgo_talisman</v>
+        <v>equip_leather_armor</v>
       </c>
       <c r="B20" t="str">
-        <v>🍂</v>
+        <v>🥋</v>
       </c>
       <c r="C20" t="str">
-        <v>합심의 황금 은행잎 부적</v>
+        <v>가죽갑옷</v>
       </c>
       <c r="D20" t="str">
         <v>장비</v>
       </c>
       <c r="E20" t="str">
-        <v>장신구 (Accessory)</v>
+        <v>갑옷 (Armor)</v>
       </c>
       <c r="F20" t="str">
-        <v>ATK +20, DEF +12, HP +40</v>
+        <v>방어력(DEF) +17, 체력(HP) +20</v>
       </c>
       <c r="G20" t="str">
-        <v>복도 제작(은행잎 10+50G)</v>
+        <v>복도 제작(보스가죽 1+농구가죽 30+50G), 림가디언(8%)</v>
       </c>
       <c r="H20" t="str">
-        <v>숭실의 교목 은행나무의 합심과 지혜가 깃든 부적</v>
+        <v>2티어 스포츠 방어구</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>equip_bronze_sword</v>
+        <v>equip_forsythia_ring</v>
       </c>
       <c r="B21" t="str">
-        <v>⚔️</v>
+        <v>🌼</v>
       </c>
       <c r="C21" t="str">
-        <v>청동검</v>
+        <v>성실의 개나리 반지</v>
       </c>
       <c r="D21" t="str">
         <v>장비</v>
       </c>
       <c r="E21" t="str">
-        <v>무기 (Weapon)</v>
+        <v>장신구 (Accessory)</v>
       </c>
       <c r="F21" t="str">
-        <v>공격력(ATK) +25</v>
+        <v>ATK +10, DEF +10, HP +20</v>
       </c>
       <c r="G21" t="str">
-        <v>복도 제작(청동심장 1+개나리 20+50G), 드래곤(20%)</v>
+        <v>복도 제작(개나리 20+30G), 보스 레이드(5%)</v>
       </c>
       <c r="H21" t="str">
-        <v>3티어 최상급 무기</v>
+        <v>숭실의 교화 개나리의 성실한 빛이 담긴 반지</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>equip_bronze_helmet</v>
+        <v>equip_ginkgo_talisman</v>
       </c>
       <c r="B22" t="str">
-        <v>🪖</v>
+        <v>🍂</v>
       </c>
       <c r="C22" t="str">
-        <v>청동투구</v>
+        <v>합심의 황금 은행잎 부적</v>
       </c>
       <c r="D22" t="str">
         <v>장비</v>
       </c>
       <c r="E22" t="str">
-        <v>투구 (Helmet)</v>
+        <v>장신구 (Accessory)</v>
       </c>
       <c r="F22" t="str">
-        <v>방어력(DEF) +14, 체력(HP) +35</v>
+        <v>ATK +20, DEF +12, HP +40</v>
       </c>
       <c r="G22" t="str">
-        <v>복도 제작(청동심장 1+개나리 10+50G), 드래곤(20%)</v>
+        <v>복도 제작(은행잎 10+50G)</v>
       </c>
       <c r="H22" t="str">
-        <v>3티어 최상급 방어구</v>
+        <v>숭실의 교목 은행나무의 합심과 지혜가 깃든 부적</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>equip_bronze_armor</v>
+        <v>equip_bronze_sword</v>
       </c>
       <c r="B23" t="str">
-        <v>🛡️</v>
+        <v>⚔️</v>
       </c>
       <c r="C23" t="str">
-        <v>청동갑옷</v>
+        <v>청동검</v>
       </c>
       <c r="D23" t="str">
         <v>장비</v>
       </c>
       <c r="E23" t="str">
+        <v>무기 (Weapon)</v>
+      </c>
+      <c r="F23" t="str">
+        <v>공격력(ATK) +25</v>
+      </c>
+      <c r="G23" t="str">
+        <v>복도 제작(청동심장 1+개나리 20+50G), 드래곤(20%), 대마왕(35%)</v>
+      </c>
+      <c r="H23" t="str">
+        <v>3티어 최상급 무기</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>equip_bronze_helmet</v>
+      </c>
+      <c r="B24" t="str">
+        <v>🪖</v>
+      </c>
+      <c r="C24" t="str">
+        <v>청동투구</v>
+      </c>
+      <c r="D24" t="str">
+        <v>장비</v>
+      </c>
+      <c r="E24" t="str">
+        <v>투구 (Helmet)</v>
+      </c>
+      <c r="F24" t="str">
+        <v>방어력(DEF) +14, 체력(HP) +35</v>
+      </c>
+      <c r="G24" t="str">
+        <v>복도 제작(청동심장 1+개나리 10+50G), 드래곤(20%), 대마왕(35%)</v>
+      </c>
+      <c r="H24" t="str">
+        <v>3티어 최상급 방어구</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>equip_bronze_armor</v>
+      </c>
+      <c r="B25" t="str">
+        <v>🛡️</v>
+      </c>
+      <c r="C25" t="str">
+        <v>청동갑옷</v>
+      </c>
+      <c r="D25" t="str">
+        <v>장비</v>
+      </c>
+      <c r="E25" t="str">
         <v>갑옷 (Armor)</v>
       </c>
-      <c r="F23" t="str">
+      <c r="F25" t="str">
         <v>방어력(DEF) +22, 체력(HP) +25</v>
       </c>
-      <c r="G23" t="str">
-        <v>복도 제작(청동심장 1+개나리 15+70G), 드래곤(20%)</v>
-      </c>
-      <c r="H23" t="str">
+      <c r="G25" t="str">
+        <v>복도 제작(청동심장 1+개나리 15+70G), 드래곤(20%), 대마왕(35%)</v>
+      </c>
+      <c r="H25" t="str">
         <v>3티어 최상급 중갑옷</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>title_perfect_exam</v>
+      </c>
+      <c r="B26" t="str">
+        <v>📚</v>
+      </c>
+      <c r="C26" t="str">
+        <v>[호칭] 시험의 제왕</v>
+      </c>
+      <c r="D26" t="str">
+        <v>호칭</v>
+      </c>
+      <c r="E26" t="str">
+        <v>칭호 (Title)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>학생 닉네임 앞 [시험의 제왕] 표기</v>
+      </c>
+      <c r="G26" t="str">
+        <v>매점 호칭 교환소 (백점만점 시험지 1장)</v>
+      </c>
+      <c r="H26" t="str">
+        <v>중간고사 대마왕 토벌자 특권 명예 호칭</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="32.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="32.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1046,30 +1126,33 @@
         <v>등급/구분</v>
       </c>
       <c r="D1" t="str">
+        <v>문제 출제 단원</v>
+      </c>
+      <c r="E1" t="str">
         <v>HP</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>ATK</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>DEF</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>오답 반격 피해</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>처치 골드</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>처치 EXP</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>확정/확률 재료 드랍 (Material Drops)</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>완제품 대박 드랍 (Rare Jackpot)</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>리스폰 주기</v>
       </c>
     </row>
@@ -1083,32 +1166,35 @@
       <c r="C2" t="str">
         <v>일반</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
+        <v>5단원 (Lesson 5)</v>
+      </c>
+      <c r="E2">
         <v>60</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>11</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>2</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>20 HP</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>8 G</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>15 EXP</v>
       </c>
-      <c r="J2" t="str" xml:space="preserve">
+      <c r="K2" t="str" xml:space="preserve">
         <v xml:space="preserve">🏀 농구공 가죽 1~2개 (100%)
 🌼 개나리 꽃잎 1개 (15% 행운)</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>-</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>15초</v>
       </c>
     </row>
@@ -1122,32 +1208,35 @@
       <c r="C3" t="str">
         <v>중급</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
+        <v>5단원 (Lesson 5)</v>
+      </c>
+      <c r="E3">
         <v>90</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>14</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>3</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>27 HP (풀피 20%)</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>15 G</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>25 EXP</v>
       </c>
-      <c r="J3" t="str" xml:space="preserve">
+      <c r="K3" t="str" xml:space="preserve">
         <v xml:space="preserve">🏀 농구공 가죽 1~2개 (100%)
 🌼 개나리 꽃잎 1개 (15% 행운)</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>-</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>20초</v>
       </c>
     </row>
@@ -1161,32 +1250,35 @@
       <c r="C4" t="str">
         <v>엘리트 보스</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="str">
+        <v>5단원 (Lesson 5)</v>
+      </c>
+      <c r="E4">
         <v>160</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>18</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>5</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>35 HP</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>35 G</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>50 EXP</v>
       </c>
-      <c r="J4" t="str" xml:space="preserve">
+      <c r="K4" t="str" xml:space="preserve">
         <v xml:space="preserve">🏀 농구공 가죽 3~5개 (100%)
 🌼 개나리 꽃잎 1개 (15% 행운)</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>🥋 가죽갑옷 완제품 1개 (8% 대박)</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>45초</v>
       </c>
     </row>
@@ -1200,32 +1292,35 @@
       <c r="C5" t="str">
         <v>일반</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="str">
+        <v>6단원 (Lesson 6)</v>
+      </c>
+      <c r="E5">
         <v>95</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>16</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>4</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>24 HP</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>14 G</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>28 EXP</v>
       </c>
-      <c r="J5" t="str" xml:space="preserve">
+      <c r="K5" t="str" xml:space="preserve">
         <v xml:space="preserve">⚽ 풋살공 가죽 1~3개 (100%)
 🌼 개나리 꽃잎 1개 (15% 행운)</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>-</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>15초</v>
       </c>
     </row>
@@ -1239,32 +1334,35 @@
       <c r="C6" t="str">
         <v>중급</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="str">
+        <v>6단원 (Lesson 6)</v>
+      </c>
+      <c r="E6">
         <v>120</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>22</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>6</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>32 HP</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>24 G</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>42 EXP</v>
       </c>
-      <c r="J6" t="str" xml:space="preserve">
+      <c r="K6" t="str" xml:space="preserve">
         <v xml:space="preserve">⚽ 풋살공 가죽 2~4개 (100%)
 🌼 개나리 꽃잎 1개 (15% 행운)</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>-</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>20초</v>
       </c>
     </row>
@@ -1278,39 +1376,42 @@
       <c r="C7" t="str">
         <v>엘리트 보스</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="str">
+        <v>6단원 (Lesson 6)</v>
+      </c>
+      <c r="E7">
         <v>190</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>28</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>8</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>42 HP</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>50 G</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>80 EXP</v>
       </c>
-      <c r="J7" t="str" xml:space="preserve">
+      <c r="K7" t="str" xml:space="preserve">
         <v xml:space="preserve">⚽ 풋살공 가죽 4~6개 (100%)
 🌼 개나리 꽃잎 1개 (15% 행운)</v>
       </c>
-      <c r="K7" t="str" xml:space="preserve">
+      <c r="L7" t="str" xml:space="preserve">
         <v xml:space="preserve">⛑️ 가죽투구 완제품 (8% 대박)
 🗡️ 가죽손잡이 세이버 (5% 대박)</v>
       </c>
-      <c r="L7" t="str">
+      <c r="M7" t="str">
         <v>45초</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1322,10 +1423,10 @@
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="32.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="54.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1359,17 +1460,17 @@
         <v>1학년 2반 1차 관문 보스 (10인 권장)</v>
       </c>
       <c r="C2" t="str">
-        <v>HP 2000 / ATK 17 / DEF 8</v>
+        <v>HP 2000 / ATK 30 / DEF 14</v>
       </c>
       <c r="D2" t="str">
         <v>🪙 +50 Gold, 🌟 +100 EXP</v>
       </c>
       <c r="E2" t="str">
-        <v>🍷/🧪 빨강/주황 물약 2~3개 확정 드랍</v>
+        <v>🍷 빨간 물약 + 🧪 주홍 물약 2~3개 확정 드랍</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">• 🟫 질긴 보스의 가죽: 1~2개 확정 (100%)
-• 나무장비(검/투구/갑옷 중 1개): 25%
+• 1티어 나무장비(검/투구/갑옷 중 1개): 25%
 • 🌼 성실의 개나리 반지: 5%</v>
       </c>
       <c r="G2" t="str">
@@ -1384,13 +1485,13 @@
         <v>1학년 2반 2차 졸업 보스 (20인 권장)</v>
       </c>
       <c r="C3" t="str">
-        <v>HP 5000 / ATK 28 / DEF 10</v>
+        <v>HP 5000 / ATK 50 / DEF 20</v>
       </c>
       <c r="D3" t="str">
         <v>🪙 +120 Gold, 🌟 +250 EXP</v>
       </c>
       <c r="E3" t="str">
-        <v>🍷/🧪 빨강/주황 물약 2~3개 확정 드랍</v>
+        <v>🍷 빨간 물약 + 🧪 주홍 물약 2~3개 확정 드랍</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">• 🥉 청동 드래곤의 심장: 1개 확정 (100%)
@@ -1401,50 +1502,53 @@
         <v>3티어 청동 장비 세트 제작 핵심 재료 공급 (2티어 완제품 지원)</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>😈 중간고사 대마왕</v>
+        <v>😈 중간고사 대마왕 (Demon King)</v>
       </c>
       <c r="B4" t="str">
         <v>축구장 서쪽 골대 (이벤트 레이드)</v>
       </c>
       <c r="C4" t="str">
-        <v>HP 999999 / ATK 150 / DEF 50 (처치 불가)</v>
+        <v>HP 7500 / ATK 86 / DEF 28</v>
       </c>
       <c r="D4" t="str">
-        <v>교사 주관 이벤트</v>
+        <v>🪙 +300 Gold, 🌟 +600 EXP</v>
       </c>
       <c r="E4" t="str">
-        <v>-</v>
-      </c>
-      <c r="F4" t="str">
-        <v>-</v>
+        <v>🧪 주홍 물약 3개 확정 + 🍷/🧪 추가 물약 2~3개 확정</v>
+      </c>
+      <c r="F4" t="str" xml:space="preserve">
+        <v xml:space="preserve">• 💯 백점만점 시험지: 1개 확정 (100% ➔ 📚 시험의 제왕 호칭 교환)
+• 3티어 청동장비(청동검/청동투구/청동갑옷 중 1종): 35% 확률 대박!
+• 🌼 성실의 개나리 반지: 5%</v>
       </c>
       <c r="G4" t="str">
-        <v>교사 관제탑에서 학기말 특별 소환 이벤트 지원</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>이벤트성 대형 보스 (대량 골드/EXP 및 부족한 청동 장비 세트 보충)</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>🐺 케르베로스</v>
+        <v>🐕 수행평가 3두마수 케르베로스</v>
       </c>
       <c r="B5" t="str">
-        <v>축구장 서쪽 골대 (이벤트 레이드)</v>
+        <v>축구장 서쪽 골대 (관문 레이드)</v>
       </c>
       <c r="C5" t="str">
-        <v>HP 999999 / ATK 150 / DEF 50 (처치 불가)</v>
+        <v>HP 8000 / ATK 90 / DEF 28</v>
       </c>
       <c r="D5" t="str">
-        <v>교사 주관 이벤트</v>
+        <v>🪙 +200 Gold, 🌟 +400 EXP</v>
       </c>
       <c r="E5" t="str">
-        <v>-</v>
-      </c>
-      <c r="F5" t="str">
-        <v>-</v>
+        <v>🍷 빨간 물약 + 🧪 주홍 물약 2~3개 확정 드랍</v>
+      </c>
+      <c r="F5" t="str" xml:space="preserve">
+        <v xml:space="preserve">• 📜 A+ 만점 수행평가지: 1개 확정 (100% ➔ 매점 25G 매각)
+• 🌼 성실의 개나리 반지: 5%</v>
       </c>
       <c r="G5" t="str">
-        <v>수행평가 시즌 특별 소환</v>
+        <v>풀청동 세트 착용 후 토벌 권장 (5~6단원 출제, 토벌 시 다음 신규 모험 구역 해금)</v>
       </c>
     </row>
   </sheetData>
@@ -1822,7 +1926,7 @@
         <v>빨간 물약</v>
       </c>
       <c r="B13" t="str">
-        <v>🧪</v>
+        <v>🍷</v>
       </c>
       <c r="C13" t="str">
         <v>소비품</v>
@@ -1848,10 +1952,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>주황 물약</v>
+        <v>주홍 물약</v>
       </c>
       <c r="B14" t="str">
-        <v>🍹</v>
+        <v>🧪</v>
       </c>
       <c r="C14" t="str">
         <v>소비품</v>
@@ -1909,4 +2013,208 @@
     <ignoredError numberStoredAsText="1" sqref="A1:I15"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G8"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="42.83203125" customWidth="1"/>
+    <col min="7" max="7" width="36.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>성장 항목 / 티어 구분</v>
+      </c>
+      <c r="B1" t="str">
+        <v>세부 구성</v>
+      </c>
+      <c r="C1" t="str">
+        <v>체력 (HP)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>공격력 (ATK)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>방어력 (DEF)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>합산 스펙 및 특징</v>
+      </c>
+      <c r="G1" t="str">
+        <v>권장 도전 목표</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>레벨 1 기본 스펙</v>
+      </c>
+      <c r="B2" t="str">
+        <v>기본 신입생</v>
+      </c>
+      <c r="C2" t="str">
+        <v>HP 100 (고정)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>ATK 10</v>
+      </c>
+      <c r="E2" t="str">
+        <v>DEF 0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>기초 스펙 (레벨업 시 HP 증가 없음, ATK +1, DEF +1)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>1반 목재/약초 채집</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>레벨 5 기본 스펙</v>
+      </c>
+      <c r="B3" t="str">
+        <v>성장 학생 (Lv.5)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>HP 100 (고정)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>ATK 14</v>
+      </c>
+      <c r="E3" t="str">
+        <v>DEF 4</v>
+      </c>
+      <c r="F3" t="str">
+        <v>순수 레벨 보너스 (+4 ATK, +4 DEF)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>농구장 일반 몬스터</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>레벨 10 기본 스펙</v>
+      </c>
+      <c r="B4" t="str">
+        <v>숙련 학생 (Lv.10)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>HP 100 (고정)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ATK 19</v>
+      </c>
+      <c r="E4" t="str">
+        <v>DEF 9</v>
+      </c>
+      <c r="F4" t="str">
+        <v>순수 레벨 보너스 (+9 ATK, +9 DEF)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>풋살장 및 보스전</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>1티어 나무 풀세트</v>
+      </c>
+      <c r="B5" t="str">
+        <v>나무검 + 나무투구 + 나무갑옷</v>
+      </c>
+      <c r="C5" t="str">
+        <v>HP +40 (총 140)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>ATK +15</v>
+      </c>
+      <c r="E5" t="str">
+        <v>DEF +23</v>
+      </c>
+      <c r="F5" t="str">
+        <v>세트 합산: ATK +15, DEF +23, HP +40</v>
+      </c>
+      <c r="G5" t="str">
+        <v>가죽 골렘 도전 (1학년 2반)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2티어 가죽 풀세트</v>
+      </c>
+      <c r="B6" t="str">
+        <v>가죽세이버 + 가죽투구 + 가죽갑옷</v>
+      </c>
+      <c r="C6" t="str">
+        <v>HP +48 (총 148)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>ATK +20</v>
+      </c>
+      <c r="E6" t="str">
+        <v>DEF +29</v>
+      </c>
+      <c r="F6" t="str">
+        <v>세트 합산: ATK +20, DEF +29, HP +48</v>
+      </c>
+      <c r="G6" t="str">
+        <v>청동 드래곤 도전 (1학년 2반)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>3티어 청동 풀세트</v>
+      </c>
+      <c r="B7" t="str">
+        <v>청동검 + 청동투구 + 청동갑옷</v>
+      </c>
+      <c r="C7" t="str">
+        <v>HP +60 (총 160)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>ATK +25</v>
+      </c>
+      <c r="E7" t="str">
+        <v>DEF +36</v>
+      </c>
+      <c r="F7" t="str">
+        <v>세트 합산: ATK +25, DEF +36, HP +60</v>
+      </c>
+      <c r="G7" t="str">
+        <v>케르베로스 &amp; 중간고사 대마왕 도전</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>풀청동 + 개나리 반지</v>
+      </c>
+      <c r="B8" t="str">
+        <v>청동 풀세트 + 성실의 개나리 반지</v>
+      </c>
+      <c r="C8" t="str">
+        <v>HP +80 (총 180)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>ATK +35</v>
+      </c>
+      <c r="E8" t="str">
+        <v>DEF +46</v>
+      </c>
+      <c r="F8" t="str">
+        <v>최상위 스펙 (합산 공+35, 방+46, 체+80)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>레이드 MVP 및 최종 관문 돌파</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add elevator pass item dropped by Golem with visual elevator status updates
</commit_message>
<xml_diff>
--- a/public/downloads/soongsil_rpg_item_drops_catalog.xlsx
+++ b/public/downloads/soongsil_rpg_item_drops_catalog.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -987,111 +987,137 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>equip_bronze_sword</v>
+        <v>equip_elevator_pass</v>
       </c>
       <c r="B23" t="str">
-        <v>⚔️</v>
+        <v>🪪</v>
       </c>
       <c r="C23" t="str">
-        <v>청동검</v>
+        <v>엘리베이터 작동권</v>
       </c>
       <c r="D23" t="str">
         <v>장비</v>
       </c>
       <c r="E23" t="str">
-        <v>무기 (Weapon)</v>
+        <v>장신구 (Accessory)</v>
       </c>
       <c r="F23" t="str">
-        <v>공격력(ATK) +25</v>
+        <v>ATK +5, DEF +5, HP +20</v>
       </c>
       <c r="G23" t="str">
-        <v>복도 제작(청동심장 1+개나리 20+50G), 드래곤(20%), 대마왕(35%)</v>
+        <v>👾 가죽 골렘 토벌(100% 확정 지급)</v>
       </c>
       <c r="H23" t="str">
-        <v>3티어 최상급 무기</v>
+        <v>중앙 엘리베이터 가동 필수 장비 (장신구 슬롯 장착 시 운동장 이동 가능)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>equip_bronze_helmet</v>
+        <v>equip_bronze_sword</v>
       </c>
       <c r="B24" t="str">
-        <v>🪖</v>
+        <v>⚔️</v>
       </c>
       <c r="C24" t="str">
-        <v>청동투구</v>
+        <v>청동검</v>
       </c>
       <c r="D24" t="str">
         <v>장비</v>
       </c>
       <c r="E24" t="str">
-        <v>투구 (Helmet)</v>
+        <v>무기 (Weapon)</v>
       </c>
       <c r="F24" t="str">
-        <v>방어력(DEF) +14, 체력(HP) +35</v>
+        <v>공격력(ATK) +25</v>
       </c>
       <c r="G24" t="str">
-        <v>복도 제작(청동심장 1+개나리 10+50G), 드래곤(20%), 대마왕(35%)</v>
+        <v>복도 제작(청동심장 1+개나리 20+50G), 드래곤(20%), 대마왕(35%)</v>
       </c>
       <c r="H24" t="str">
-        <v>3티어 최상급 방어구</v>
+        <v>3티어 최상급 무기</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>equip_bronze_armor</v>
+        <v>equip_bronze_helmet</v>
       </c>
       <c r="B25" t="str">
-        <v>🛡️</v>
+        <v>🪖</v>
       </c>
       <c r="C25" t="str">
-        <v>청동갑옷</v>
+        <v>청동투구</v>
       </c>
       <c r="D25" t="str">
         <v>장비</v>
       </c>
       <c r="E25" t="str">
-        <v>갑옷 (Armor)</v>
+        <v>투구 (Helmet)</v>
       </c>
       <c r="F25" t="str">
-        <v>방어력(DEF) +22, 체력(HP) +25</v>
+        <v>방어력(DEF) +14, 체력(HP) +35</v>
       </c>
       <c r="G25" t="str">
-        <v>복도 제작(청동심장 1+개나리 15+70G), 드래곤(20%), 대마왕(35%)</v>
+        <v>복도 제작(청동심장 1+개나리 10+50G), 드래곤(20%), 대마왕(35%)</v>
       </c>
       <c r="H25" t="str">
-        <v>3티어 최상급 중갑옷</v>
+        <v>3티어 최상급 방어구</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>equip_bronze_armor</v>
+      </c>
+      <c r="B26" t="str">
+        <v>🛡️</v>
+      </c>
+      <c r="C26" t="str">
+        <v>청동갑옷</v>
+      </c>
+      <c r="D26" t="str">
+        <v>장비</v>
+      </c>
+      <c r="E26" t="str">
+        <v>갑옷 (Armor)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>방어력(DEF) +22, 체력(HP) +25</v>
+      </c>
+      <c r="G26" t="str">
+        <v>복도 제작(청동심장 1+개나리 15+70G), 드래곤(20%), 대마왕(35%)</v>
+      </c>
+      <c r="H26" t="str">
+        <v>3티어 최상급 중갑옷</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>title_perfect_exam</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B27" t="str">
         <v>📚</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C27" t="str">
         <v>[호칭] 시험의 제왕</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D27" t="str">
         <v>호칭</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E27" t="str">
         <v>칭호 (Title)</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F27" t="str">
         <v>학생 닉네임 앞 [시험의 제왕] 표기</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G27" t="str">
         <v>매점 호칭 교환소 (백점만점 시험지 1장)</v>
       </c>
-      <c r="H26" t="str">
+      <c r="H27" t="str">
         <v>중간고사 대마왕 토벌자 특권 명예 호칭</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1470,11 +1496,12 @@
       </c>
       <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">• 🟫 질긴 보스의 가죽: 1~2개 확정 (100%)
+• 🪪 엘리베이터 작동권: 100% 확정 지급
 • 1티어 나무장비(검/투구/갑옷 중 1개): 25%
 • 🌼 성실의 개나리 반지: 5%</v>
       </c>
       <c r="G2" t="str">
-        <v>🎉 토벌 시 중앙 엘리베이터 점검 완료 ➔ 10G로 지상 운동장 개방!</v>
+        <v>🎉 토벌 시 [🪪 엘리베이터 작동권] 획득! ➔ 장신구 슬롯 장착 후 10G로 지상 운동장 가동!</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">

</xml_diff>